<commit_message>
remove RdataTmp files + update xlsx files + update script
</commit_message>
<xml_diff>
--- a/cls.var_AMR_EHPAD_FQ_R.xlsx
+++ b/cls.var_AMR_EHPAD_FQ_R.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
   <si>
     <t xml:space="preserve">variable</t>
   </si>
@@ -32,15 +32,18 @@
     <t xml:space="preserve">log_AMC_EHPAD_macrolides</t>
   </si>
   <si>
+    <t xml:space="preserve">cluster_2</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_AMC_EHPAD_penicillines</t>
   </si>
   <si>
-    <t xml:space="preserve">cluster_2</t>
-  </si>
-  <si>
     <t xml:space="preserve">log_AMC_EHPAD_tetracyclines</t>
   </si>
   <si>
+    <t xml:space="preserve">cluster_3</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_AMC_EHPAD_totale</t>
   </si>
   <si>
@@ -65,6 +68,9 @@
     <t xml:space="preserve">log_AMC_ville_penicillines</t>
   </si>
   <si>
+    <t xml:space="preserve">cluster_4</t>
+  </si>
+  <si>
     <t xml:space="preserve">log_AMC_ville_tetracyclines</t>
   </si>
   <si>
@@ -80,6 +86,9 @@
     <t xml:space="preserve">log_AMC_ville_tot_except_FQ</t>
   </si>
   <si>
+    <t xml:space="preserve">prescri_1</t>
+  </si>
+  <si>
     <t xml:space="preserve">AMR_animaux_production_C3G_R</t>
   </si>
   <si>
@@ -92,16 +101,10 @@
     <t xml:space="preserve">veto_by_CV</t>
   </si>
   <si>
-    <t xml:space="preserve">cluster_3</t>
-  </si>
-  <si>
     <t xml:space="preserve">veto_by_carni</t>
   </si>
   <si>
     <t xml:space="preserve">tx_possession_chats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cluster_4</t>
   </si>
   <si>
     <t xml:space="preserve">log_UGB_density_bovine_all</t>
@@ -510,15 +513,15 @@
         <v>5</v>
       </c>
       <c r="B4" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B5" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -526,44 +529,44 @@
         <v>8</v>
       </c>
       <c r="B6" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B10" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
         <v>3</v>
@@ -571,79 +574,79 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B15" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
         <v>18</v>
-      </c>
-      <c r="B16" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B17" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B19" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B20" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B21" t="s">
         <v>3</v>
@@ -651,34 +654,34 @@
     </row>
     <row r="22">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B22" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B24" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -686,7 +689,7 @@
         <v>30</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27">
@@ -694,7 +697,7 @@
         <v>31</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="28">
@@ -702,7 +705,7 @@
         <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="29">
@@ -710,7 +713,7 @@
         <v>33</v>
       </c>
       <c r="B29" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="30">
@@ -718,7 +721,7 @@
         <v>34</v>
       </c>
       <c r="B30" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -726,7 +729,7 @@
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
     </row>
     <row r="32">
@@ -734,7 +737,7 @@
         <v>36</v>
       </c>
       <c r="B32" t="s">
-        <v>29</v>
+        <v>9</v>
       </c>
     </row>
     <row r="33">
@@ -742,7 +745,7 @@
         <v>37</v>
       </c>
       <c r="B33" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -750,7 +753,7 @@
         <v>38</v>
       </c>
       <c r="B34" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="35">
@@ -758,7 +761,7 @@
         <v>39</v>
       </c>
       <c r="B35" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
@@ -774,7 +777,7 @@
         <v>41</v>
       </c>
       <c r="B37" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38">
@@ -782,7 +785,7 @@
         <v>42</v>
       </c>
       <c r="B38" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="39">
@@ -790,7 +793,7 @@
         <v>43</v>
       </c>
       <c r="B39" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
     <row r="40">
@@ -798,7 +801,7 @@
         <v>44</v>
       </c>
       <c r="B40" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="41">
@@ -814,6 +817,14 @@
         <v>46</v>
       </c>
       <c r="B42" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>47</v>
+      </c>
+      <c r="B43" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>